<commit_message>
Correção de erro de digitação
</commit_message>
<xml_diff>
--- a/relatorios/relatorio_turma.xlsx
+++ b/relatorios/relatorio_turma.xlsx
@@ -8,11 +8,11 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Relatório_Turma" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Estatísticas" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Sheet!$A$1:$G$11</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Relatório_Turma!$A$1:$G$11</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -205,16 +205,16 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -501,263 +501,263 @@
   <dimension ref="A1:G11"/>
   <sheetFormatPr defaultColWidth="8.453125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="21.84"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12.46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12.55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="0" width="12.46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="16.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="21.84"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12.55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="1" width="12.46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="16.83"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="2" t="n">
+      <c r="B2" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="C2" s="2" t="n">
+      <c r="C2" s="3" t="n">
         <v>8.5</v>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="D2" s="3" t="n">
         <v>9.5</v>
       </c>
-      <c r="E2" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="F2" s="2" t="n">
+      <c r="E2" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="F2" s="3" t="n">
         <v>8.75</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="3" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="2" t="n">
+      <c r="B3" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="C3" s="2" t="n">
+      <c r="C3" s="3" t="n">
         <v>6.5</v>
       </c>
-      <c r="D3" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="E3" s="2" t="n">
+      <c r="D3" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="E3" s="3" t="n">
         <v>7.5</v>
       </c>
-      <c r="F3" s="2" t="n">
+      <c r="F3" s="3" t="n">
         <v>7.25</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="3" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="2" t="n">
+      <c r="B4" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="C4" s="2" t="n">
+      <c r="C4" s="3" t="n">
         <v>9.5</v>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="D4" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="E4" s="2" t="n">
+      <c r="E4" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="F4" s="3" t="n">
         <v>9.62</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="G4" s="3" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="2" t="n">
+      <c r="B5" s="3" t="n">
         <v>5.5</v>
       </c>
-      <c r="C5" s="2" t="n">
+      <c r="C5" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="D5" s="2" t="n">
+      <c r="D5" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="E5" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="F5" s="2" t="n">
+      <c r="F5" s="3" t="n">
         <v>5.88</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="G5" s="3" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="2" t="n">
+      <c r="B6" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="C6" s="2" t="n">
+      <c r="C6" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="D6" s="2" t="n">
+      <c r="D6" s="3" t="n">
         <v>4.5</v>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="E6" s="3" t="n">
         <v>6.5</v>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="F6" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="G6" s="3" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="C7" s="2" t="n">
+      <c r="B7" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="C7" s="3" t="n">
         <v>7.5</v>
       </c>
-      <c r="D7" s="2" t="n">
+      <c r="D7" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="E7" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="F7" s="2" t="n">
+      <c r="F7" s="3" t="n">
         <v>7.88</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="G7" s="3" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="2" t="n">
+      <c r="B8" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="C8" s="2" t="n">
+      <c r="C8" s="3" t="n">
         <v>5.5</v>
       </c>
-      <c r="D8" s="2" t="n">
+      <c r="D8" s="3" t="n">
         <v>6.5</v>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="E8" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="F8" s="2" t="n">
+      <c r="F8" s="3" t="n">
         <v>5.5</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="G8" s="3" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="2" t="n">
+      <c r="B9" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="C9" s="2" t="n">
+      <c r="C9" s="3" t="n">
         <v>4.5</v>
       </c>
-      <c r="D9" s="2" t="n">
+      <c r="D9" s="3" t="n">
         <v>6.5</v>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="E9" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="F9" s="2" t="n">
+      <c r="F9" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="G9" s="3" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="2" t="n">
+      <c r="B10" s="3" t="n">
         <v>7.5</v>
       </c>
-      <c r="C10" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="D10" s="2" t="n">
+      <c r="C10" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="D10" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="E10" s="2" t="n">
+      <c r="E10" s="3" t="n">
         <v>8.5</v>
       </c>
-      <c r="F10" s="2" t="n">
+      <c r="F10" s="3" t="n">
         <v>7.5</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="G10" s="3" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B11" s="2" t="n">
+      <c r="B11" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="C11" s="2" t="n">
+      <c r="C11" s="3" t="n">
         <v>8.5</v>
       </c>
-      <c r="D11" s="2" t="n">
+      <c r="D11" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="E11" s="2" t="n">
+      <c r="E11" s="3" t="n">
         <v>9.5</v>
       </c>
-      <c r="F11" s="2" t="n">
+      <c r="F11" s="3" t="n">
         <v>9.25</v>
       </c>
-      <c r="G11" s="2" t="s">
+      <c r="G11" s="3" t="s">
         <v>8</v>
       </c>
     </row>
@@ -781,60 +781,64 @@
   </sheetPr>
   <dimension ref="A1:B7"/>
   <sheetFormatPr defaultColWidth="8.453125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14.76"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13.19"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B2" s="0" t="n">
+      <c r="B2" s="3" t="n">
         <v>7.06</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B3" s="0" t="n">
+      <c r="B3" s="3" t="n">
         <v>9.62</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B4" s="0" t="n">
+      <c r="B4" s="3" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="0" t="n">
+      <c r="B5" s="3" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="0" t="n">
+      <c r="B6" s="3" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B7" s="0" t="n">
+      <c r="B7" s="3" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>